<commit_message>
Yeni formlar oluşturup kodlarda denk geldiğim bir kaç hatayı düzelltim artık yazıcılar tablosunda is_Deleted diye bir sütun var ve yazıcıları sildiğinizde sadece size gözükmez hale gelir fakat istediğiniz zaman silinenler bölümü ekleyeceğim ordan geri döndürülebilir olucak
</commit_message>
<xml_diff>
--- a/db_backups/InkWatchDbTasarım Şeması.xlsx
+++ b/db_backups/InkWatchDbTasarım Şeması.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
   <si>
     <t>tbl_brands</t>
   </si>
@@ -70,9 +70,6 @@
     <t>model_logo</t>
   </si>
   <si>
-    <t>part_type_explanation</t>
-  </si>
-  <si>
     <t>printer_id</t>
   </si>
   <si>
@@ -82,10 +79,113 @@
     <t>printer_owner</t>
   </si>
   <si>
-    <t>printer_crash_log</t>
-  </si>
-  <si>
-    <t>printer_changepart_log</t>
+    <t>explanation_id</t>
+  </si>
+  <si>
+    <t>tbl_explanations</t>
+  </si>
+  <si>
+    <t>explation_id</t>
+  </si>
+  <si>
+    <t>explation_text</t>
+  </si>
+  <si>
+    <t>tbl_printer_logs</t>
+  </si>
+  <si>
+    <t>log_id (PK)</t>
+  </si>
+  <si>
+    <t>printer_id (FK)</t>
+  </si>
+  <si>
+    <t>log_date</t>
+  </si>
+  <si>
+    <t>error_code</t>
+  </si>
+  <si>
+    <t>error_description</t>
+  </si>
+  <si>
+    <t>resolved</t>
+  </si>
+  <si>
+    <t>resolved_date</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>technician_id</t>
+  </si>
+  <si>
+    <t>log_id</t>
+  </si>
+  <si>
+    <t>printer_sn</t>
+  </si>
+  <si>
+    <t>brand_id (primary_key)</t>
+  </si>
+  <si>
+    <t>model_id (primary_key)</t>
+  </si>
+  <si>
+    <t>brand_id (foreign_key)</t>
+  </si>
+  <si>
+    <t>part_type_id (primary_key)</t>
+  </si>
+  <si>
+    <t>compatible_devices (foreign_key)</t>
+  </si>
+  <si>
+    <t>tbl_users</t>
+  </si>
+  <si>
+    <t>user_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">username </t>
+  </si>
+  <si>
+    <t xml:space="preserve">password_hash </t>
+  </si>
+  <si>
+    <t xml:space="preserve">full_name </t>
+  </si>
+  <si>
+    <t xml:space="preserve">email </t>
+  </si>
+  <si>
+    <t>role</t>
+  </si>
+  <si>
+    <t>is_active</t>
+  </si>
+  <si>
+    <t>created_at</t>
+  </si>
+  <si>
+    <t>INSERT INTO tbl_users (username, password_hash, full_name, email, role)
+VALUES 
+('admin', SHA2('admin123', 256), 'Sistem Yöneticisi', 'admin@example.com', 'admin'),
+('mehmet', SHA2('mehmet123', 256), 'Mehmet Yılmaz', 'mehmet@example.com', 'user');</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CREATE TABLE tbl_users (
+    user_id INT AUTO_INCREMENT PRIMARY KEY,
+    username VARCHAR(50) NOT NULL UNIQUE,
+    password_hash VARCHAR(255) NOT NULL,
+    full_name VARCHAR(100),
+    email VARCHAR(100),
+    role ENUM('admin', 'user', 'viewer') DEFAULT 'user',
+    is_active BOOLEAN DEFAULT TRUE,
+    created_at TIMESTAMP DEFAULT CURRENT_TIMESTAMP
+);
+</t>
   </si>
 </sst>
 </file>
@@ -205,7 +305,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -232,6 +332,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="İyi" xfId="1" builtinId="26"/>
@@ -254,147 +363,1260 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1714500</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1762125</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>219075</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="5" name="Dirsek Bağlayıcısı 4"/>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Serbest Form 8"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1714500" y="542925"/>
-          <a:ext cx="2066925" cy="476250"/>
+          <a:off x="5362575" y="466725"/>
+          <a:ext cx="1866900" cy="1257300"/>
         </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst>
-            <a:gd name="adj1" fmla="val 37558"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst>
+            <a:gd name="connsiteX0" fmla="*/ 1866900 w 1866900"/>
+            <a:gd name="connsiteY0" fmla="*/ 1257300 h 1257300"/>
+            <a:gd name="connsiteX1" fmla="*/ 1352550 w 1866900"/>
+            <a:gd name="connsiteY1" fmla="*/ 1238250 h 1257300"/>
+            <a:gd name="connsiteX2" fmla="*/ 1285875 w 1866900"/>
+            <a:gd name="connsiteY2" fmla="*/ 1209675 h 1257300"/>
+            <a:gd name="connsiteX3" fmla="*/ 1181100 w 1866900"/>
+            <a:gd name="connsiteY3" fmla="*/ 1162050 h 1257300"/>
+            <a:gd name="connsiteX4" fmla="*/ 1152525 w 1866900"/>
+            <a:gd name="connsiteY4" fmla="*/ 1152525 h 1257300"/>
+            <a:gd name="connsiteX5" fmla="*/ 1123950 w 1866900"/>
+            <a:gd name="connsiteY5" fmla="*/ 1133475 h 1257300"/>
+            <a:gd name="connsiteX6" fmla="*/ 1057275 w 1866900"/>
+            <a:gd name="connsiteY6" fmla="*/ 1104900 h 1257300"/>
+            <a:gd name="connsiteX7" fmla="*/ 990600 w 1866900"/>
+            <a:gd name="connsiteY7" fmla="*/ 1038225 h 1257300"/>
+            <a:gd name="connsiteX8" fmla="*/ 952500 w 1866900"/>
+            <a:gd name="connsiteY8" fmla="*/ 1000125 h 1257300"/>
+            <a:gd name="connsiteX9" fmla="*/ 923925 w 1866900"/>
+            <a:gd name="connsiteY9" fmla="*/ 962025 h 1257300"/>
+            <a:gd name="connsiteX10" fmla="*/ 866775 w 1866900"/>
+            <a:gd name="connsiteY10" fmla="*/ 923925 h 1257300"/>
+            <a:gd name="connsiteX11" fmla="*/ 838200 w 1866900"/>
+            <a:gd name="connsiteY11" fmla="*/ 885825 h 1257300"/>
+            <a:gd name="connsiteX12" fmla="*/ 819150 w 1866900"/>
+            <a:gd name="connsiteY12" fmla="*/ 847725 h 1257300"/>
+            <a:gd name="connsiteX13" fmla="*/ 790575 w 1866900"/>
+            <a:gd name="connsiteY13" fmla="*/ 800100 h 1257300"/>
+            <a:gd name="connsiteX14" fmla="*/ 742950 w 1866900"/>
+            <a:gd name="connsiteY14" fmla="*/ 733425 h 1257300"/>
+            <a:gd name="connsiteX15" fmla="*/ 723900 w 1866900"/>
+            <a:gd name="connsiteY15" fmla="*/ 704850 h 1257300"/>
+            <a:gd name="connsiteX16" fmla="*/ 695325 w 1866900"/>
+            <a:gd name="connsiteY16" fmla="*/ 609600 h 1257300"/>
+            <a:gd name="connsiteX17" fmla="*/ 676275 w 1866900"/>
+            <a:gd name="connsiteY17" fmla="*/ 561975 h 1257300"/>
+            <a:gd name="connsiteX18" fmla="*/ 666750 w 1866900"/>
+            <a:gd name="connsiteY18" fmla="*/ 523875 h 1257300"/>
+            <a:gd name="connsiteX19" fmla="*/ 657225 w 1866900"/>
+            <a:gd name="connsiteY19" fmla="*/ 495300 h 1257300"/>
+            <a:gd name="connsiteX20" fmla="*/ 647700 w 1866900"/>
+            <a:gd name="connsiteY20" fmla="*/ 428625 h 1257300"/>
+            <a:gd name="connsiteX21" fmla="*/ 638175 w 1866900"/>
+            <a:gd name="connsiteY21" fmla="*/ 342900 h 1257300"/>
+            <a:gd name="connsiteX22" fmla="*/ 628650 w 1866900"/>
+            <a:gd name="connsiteY22" fmla="*/ 285750 h 1257300"/>
+            <a:gd name="connsiteX23" fmla="*/ 609600 w 1866900"/>
+            <a:gd name="connsiteY23" fmla="*/ 257175 h 1257300"/>
+            <a:gd name="connsiteX24" fmla="*/ 600075 w 1866900"/>
+            <a:gd name="connsiteY24" fmla="*/ 228600 h 1257300"/>
+            <a:gd name="connsiteX25" fmla="*/ 533400 w 1866900"/>
+            <a:gd name="connsiteY25" fmla="*/ 133350 h 1257300"/>
+            <a:gd name="connsiteX26" fmla="*/ 514350 w 1866900"/>
+            <a:gd name="connsiteY26" fmla="*/ 104775 h 1257300"/>
+            <a:gd name="connsiteX27" fmla="*/ 457200 w 1866900"/>
+            <a:gd name="connsiteY27" fmla="*/ 57150 h 1257300"/>
+            <a:gd name="connsiteX28" fmla="*/ 438150 w 1866900"/>
+            <a:gd name="connsiteY28" fmla="*/ 28575 h 1257300"/>
+            <a:gd name="connsiteX29" fmla="*/ 409575 w 1866900"/>
+            <a:gd name="connsiteY29" fmla="*/ 19050 h 1257300"/>
+            <a:gd name="connsiteX30" fmla="*/ 381000 w 1866900"/>
+            <a:gd name="connsiteY30" fmla="*/ 0 h 1257300"/>
+            <a:gd name="connsiteX31" fmla="*/ 104775 w 1866900"/>
+            <a:gd name="connsiteY31" fmla="*/ 9525 h 1257300"/>
+            <a:gd name="connsiteX32" fmla="*/ 57150 w 1866900"/>
+            <a:gd name="connsiteY32" fmla="*/ 47625 h 1257300"/>
+            <a:gd name="connsiteX33" fmla="*/ 28575 w 1866900"/>
+            <a:gd name="connsiteY33" fmla="*/ 66675 h 1257300"/>
+            <a:gd name="connsiteX34" fmla="*/ 0 w 1866900"/>
+            <a:gd name="connsiteY34" fmla="*/ 95250 h 1257300"/>
+          </a:gdLst>
+          <a:ahLst/>
+          <a:cxnLst>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX0" y="connsiteY0"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX1" y="connsiteY1"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX2" y="connsiteY2"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX3" y="connsiteY3"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX4" y="connsiteY4"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX5" y="connsiteY5"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX6" y="connsiteY6"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX7" y="connsiteY7"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX8" y="connsiteY8"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX9" y="connsiteY9"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX10" y="connsiteY10"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX11" y="connsiteY11"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX12" y="connsiteY12"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX13" y="connsiteY13"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX14" y="connsiteY14"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX15" y="connsiteY15"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX16" y="connsiteY16"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX17" y="connsiteY17"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX18" y="connsiteY18"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX19" y="connsiteY19"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX20" y="connsiteY20"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX21" y="connsiteY21"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX22" y="connsiteY22"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX23" y="connsiteY23"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX24" y="connsiteY24"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX25" y="connsiteY25"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX26" y="connsiteY26"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX27" y="connsiteY27"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX28" y="connsiteY28"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX29" y="connsiteY29"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX30" y="connsiteY30"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX31" y="connsiteY31"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX32" y="connsiteY32"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX33" y="connsiteY33"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX34" y="connsiteY34"/>
+            </a:cxn>
+          </a:cxnLst>
+          <a:rect l="l" t="t" r="r" b="b"/>
+          <a:pathLst>
+            <a:path w="1866900" h="1257300">
+              <a:moveTo>
+                <a:pt x="1866900" y="1257300"/>
+              </a:moveTo>
+              <a:cubicBezTo>
+                <a:pt x="1829507" y="1256430"/>
+                <a:pt x="1488747" y="1257707"/>
+                <a:pt x="1352550" y="1238250"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1328703" y="1234843"/>
+                <a:pt x="1307219" y="1218213"/>
+                <a:pt x="1285875" y="1209675"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1091020" y="1131733"/>
+                <a:pt x="1356709" y="1249855"/>
+                <a:pt x="1181100" y="1162050"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1172120" y="1157560"/>
+                <a:pt x="1161505" y="1157015"/>
+                <a:pt x="1152525" y="1152525"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1142286" y="1147405"/>
+                <a:pt x="1134189" y="1138595"/>
+                <a:pt x="1123950" y="1133475"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1093172" y="1118086"/>
+                <a:pt x="1088421" y="1130383"/>
+                <a:pt x="1057275" y="1104900"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1032949" y="1084997"/>
+                <a:pt x="1012825" y="1060450"/>
+                <a:pt x="990600" y="1038225"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="977900" y="1025525"/>
+                <a:pt x="963276" y="1014493"/>
+                <a:pt x="952500" y="1000125"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="942975" y="987425"/>
+                <a:pt x="935790" y="972572"/>
+                <a:pt x="923925" y="962025"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="906813" y="946814"/>
+                <a:pt x="880512" y="942241"/>
+                <a:pt x="866775" y="923925"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="857250" y="911225"/>
+                <a:pt x="846614" y="899287"/>
+                <a:pt x="838200" y="885825"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="830675" y="873784"/>
+                <a:pt x="826046" y="860137"/>
+                <a:pt x="819150" y="847725"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="810159" y="831541"/>
+                <a:pt x="800387" y="815799"/>
+                <a:pt x="790575" y="800100"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="768127" y="764184"/>
+                <a:pt x="770894" y="772546"/>
+                <a:pt x="742950" y="733425"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="736296" y="724110"/>
+                <a:pt x="728549" y="715311"/>
+                <a:pt x="723900" y="704850"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="694458" y="638606"/>
+                <a:pt x="713796" y="665013"/>
+                <a:pt x="695325" y="609600"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="689918" y="593380"/>
+                <a:pt x="681682" y="578195"/>
+                <a:pt x="676275" y="561975"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="672135" y="549556"/>
+                <a:pt x="670346" y="536462"/>
+                <a:pt x="666750" y="523875"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="663992" y="514221"/>
+                <a:pt x="660400" y="504825"/>
+                <a:pt x="657225" y="495300"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="654050" y="473075"/>
+                <a:pt x="650485" y="450902"/>
+                <a:pt x="647700" y="428625"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="644134" y="400096"/>
+                <a:pt x="641975" y="371399"/>
+                <a:pt x="638175" y="342900"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="635623" y="323757"/>
+                <a:pt x="634757" y="304072"/>
+                <a:pt x="628650" y="285750"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="625030" y="274890"/>
+                <a:pt x="614720" y="267414"/>
+                <a:pt x="609600" y="257175"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="605110" y="248195"/>
+                <a:pt x="604951" y="237377"/>
+                <a:pt x="600075" y="228600"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="578178" y="189185"/>
+                <a:pt x="558372" y="168310"/>
+                <a:pt x="533400" y="133350"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="526746" y="124035"/>
+                <a:pt x="521679" y="113569"/>
+                <a:pt x="514350" y="104775"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="491431" y="77273"/>
+                <a:pt x="485297" y="75881"/>
+                <a:pt x="457200" y="57150"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="450850" y="47625"/>
+                <a:pt x="447089" y="35726"/>
+                <a:pt x="438150" y="28575"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="430310" y="22303"/>
+                <a:pt x="418555" y="23540"/>
+                <a:pt x="409575" y="19050"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="399336" y="13930"/>
+                <a:pt x="390525" y="6350"/>
+                <a:pt x="381000" y="0"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="288925" y="3175"/>
+                <a:pt x="196725" y="3778"/>
+                <a:pt x="104775" y="9525"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="65216" y="11997"/>
+                <a:pt x="81910" y="22865"/>
+                <a:pt x="57150" y="47625"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="49055" y="55720"/>
+                <a:pt x="37369" y="59346"/>
+                <a:pt x="28575" y="66675"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="18227" y="75299"/>
+                <a:pt x="0" y="95250"/>
+                <a:pt x="0" y="95250"/>
+              </a:cubicBezTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:noFill/>
       </xdr:spPr>
       <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
         </a:lnRef>
-        <a:fillRef idx="0">
+        <a:fillRef idx="1">
           <a:schemeClr val="accent1"/>
         </a:fillRef>
         <a:effectRef idx="0">
           <a:schemeClr val="accent1"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
+          <a:schemeClr val="lt1"/>
         </a:fontRef>
       </xdr:style>
-    </xdr:cxnSp>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="tr-TR" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1552575</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1695450</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>342900</xdr:rowOff>
+      <xdr:rowOff>228600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>219075</xdr:rowOff>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="7" name="Dirsek Bağlayıcısı 6"/>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Serbest Form 9"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5153025" y="742950"/>
-          <a:ext cx="5762625" cy="276225"/>
+          <a:off x="1695450" y="628650"/>
+          <a:ext cx="1990725" cy="352425"/>
         </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst>
-            <a:gd name="adj1" fmla="val 84050"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst>
+            <a:gd name="connsiteX0" fmla="*/ 0 w 1990725"/>
+            <a:gd name="connsiteY0" fmla="*/ 0 h 352425"/>
+            <a:gd name="connsiteX1" fmla="*/ 1114425 w 1990725"/>
+            <a:gd name="connsiteY1" fmla="*/ 28575 h 352425"/>
+            <a:gd name="connsiteX2" fmla="*/ 1209675 w 1990725"/>
+            <a:gd name="connsiteY2" fmla="*/ 171450 h 352425"/>
+            <a:gd name="connsiteX3" fmla="*/ 1228725 w 1990725"/>
+            <a:gd name="connsiteY3" fmla="*/ 200025 h 352425"/>
+            <a:gd name="connsiteX4" fmla="*/ 1276350 w 1990725"/>
+            <a:gd name="connsiteY4" fmla="*/ 257175 h 352425"/>
+            <a:gd name="connsiteX5" fmla="*/ 1304925 w 1990725"/>
+            <a:gd name="connsiteY5" fmla="*/ 266700 h 352425"/>
+            <a:gd name="connsiteX6" fmla="*/ 1371600 w 1990725"/>
+            <a:gd name="connsiteY6" fmla="*/ 295275 h 352425"/>
+            <a:gd name="connsiteX7" fmla="*/ 1400175 w 1990725"/>
+            <a:gd name="connsiteY7" fmla="*/ 304800 h 352425"/>
+            <a:gd name="connsiteX8" fmla="*/ 1438275 w 1990725"/>
+            <a:gd name="connsiteY8" fmla="*/ 314325 h 352425"/>
+            <a:gd name="connsiteX9" fmla="*/ 1476375 w 1990725"/>
+            <a:gd name="connsiteY9" fmla="*/ 333375 h 352425"/>
+            <a:gd name="connsiteX10" fmla="*/ 1581150 w 1990725"/>
+            <a:gd name="connsiteY10" fmla="*/ 342900 h 352425"/>
+            <a:gd name="connsiteX11" fmla="*/ 1676400 w 1990725"/>
+            <a:gd name="connsiteY11" fmla="*/ 352425 h 352425"/>
+            <a:gd name="connsiteX12" fmla="*/ 1990725 w 1990725"/>
+            <a:gd name="connsiteY12" fmla="*/ 342900 h 352425"/>
+          </a:gdLst>
+          <a:ahLst/>
+          <a:cxnLst>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX0" y="connsiteY0"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX1" y="connsiteY1"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX2" y="connsiteY2"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX3" y="connsiteY3"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX4" y="connsiteY4"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX5" y="connsiteY5"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX6" y="connsiteY6"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX7" y="connsiteY7"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX8" y="connsiteY8"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX9" y="connsiteY9"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX10" y="connsiteY10"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX11" y="connsiteY11"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX12" y="connsiteY12"/>
+            </a:cxn>
+          </a:cxnLst>
+          <a:rect l="l" t="t" r="r" b="b"/>
+          <a:pathLst>
+            <a:path w="1990725" h="352425">
+              <a:moveTo>
+                <a:pt x="0" y="0"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="1114425" y="28575"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="1209675" y="171450"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="1228725" y="200025"/>
+              </a:lnTo>
+              <a:cubicBezTo>
+                <a:pt x="1242782" y="221110"/>
+                <a:pt x="1254348" y="242507"/>
+                <a:pt x="1276350" y="257175"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1284704" y="262744"/>
+                <a:pt x="1295945" y="262210"/>
+                <a:pt x="1304925" y="266700"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1382261" y="305368"/>
+                <a:pt x="1279090" y="268844"/>
+                <a:pt x="1371600" y="295275"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1381254" y="298033"/>
+                <a:pt x="1390521" y="302042"/>
+                <a:pt x="1400175" y="304800"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1412762" y="308396"/>
+                <a:pt x="1426018" y="309728"/>
+                <a:pt x="1438275" y="314325"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1451570" y="319311"/>
+                <a:pt x="1462452" y="330590"/>
+                <a:pt x="1476375" y="333375"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1510763" y="340253"/>
+                <a:pt x="1546239" y="339575"/>
+                <a:pt x="1581150" y="342900"/>
+              </a:cubicBezTo>
+              <a:lnTo>
+                <a:pt x="1676400" y="352425"/>
+              </a:lnTo>
+              <a:cubicBezTo>
+                <a:pt x="1971670" y="342583"/>
+                <a:pt x="1866847" y="342900"/>
+                <a:pt x="1990725" y="342900"/>
+              </a:cubicBezTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:noFill/>
       </xdr:spPr>
       <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
         </a:lnRef>
-        <a:fillRef idx="0">
+        <a:fillRef idx="1">
           <a:schemeClr val="accent1"/>
         </a:fillRef>
         <a:effectRef idx="0">
           <a:schemeClr val="accent1"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
+          <a:schemeClr val="lt1"/>
         </a:fontRef>
       </xdr:style>
-    </xdr:cxnSp>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="tr-TR" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1704975</xdr:colOff>
+      <xdr:colOff>2143125</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>219075</xdr:rowOff>
+      <xdr:rowOff>171103</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
+      <xdr:colOff>190500</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>238125</xdr:rowOff>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="19" name="Dirsek Bağlayıcısı 18"/>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Serbest Form 10"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8905875" y="619125"/>
-          <a:ext cx="2057400" cy="819150"/>
+          <a:off x="9344025" y="571153"/>
+          <a:ext cx="2124075" cy="809972"/>
         </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
+        <a:custGeom>
           <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
+          <a:gdLst>
+            <a:gd name="connsiteX0" fmla="*/ 2124075 w 2124075"/>
+            <a:gd name="connsiteY0" fmla="*/ 809972 h 809972"/>
+            <a:gd name="connsiteX1" fmla="*/ 1743075 w 2124075"/>
+            <a:gd name="connsiteY1" fmla="*/ 800447 h 809972"/>
+            <a:gd name="connsiteX2" fmla="*/ 1714500 w 2124075"/>
+            <a:gd name="connsiteY2" fmla="*/ 790922 h 809972"/>
+            <a:gd name="connsiteX3" fmla="*/ 1628775 w 2124075"/>
+            <a:gd name="connsiteY3" fmla="*/ 771872 h 809972"/>
+            <a:gd name="connsiteX4" fmla="*/ 1552575 w 2124075"/>
+            <a:gd name="connsiteY4" fmla="*/ 752822 h 809972"/>
+            <a:gd name="connsiteX5" fmla="*/ 1209675 w 2124075"/>
+            <a:gd name="connsiteY5" fmla="*/ 733772 h 809972"/>
+            <a:gd name="connsiteX6" fmla="*/ 1171575 w 2124075"/>
+            <a:gd name="connsiteY6" fmla="*/ 724247 h 809972"/>
+            <a:gd name="connsiteX7" fmla="*/ 1095375 w 2124075"/>
+            <a:gd name="connsiteY7" fmla="*/ 714722 h 809972"/>
+            <a:gd name="connsiteX8" fmla="*/ 1028700 w 2124075"/>
+            <a:gd name="connsiteY8" fmla="*/ 705197 h 809972"/>
+            <a:gd name="connsiteX9" fmla="*/ 952500 w 2124075"/>
+            <a:gd name="connsiteY9" fmla="*/ 667097 h 809972"/>
+            <a:gd name="connsiteX10" fmla="*/ 895350 w 2124075"/>
+            <a:gd name="connsiteY10" fmla="*/ 609947 h 809972"/>
+            <a:gd name="connsiteX11" fmla="*/ 876300 w 2124075"/>
+            <a:gd name="connsiteY11" fmla="*/ 581372 h 809972"/>
+            <a:gd name="connsiteX12" fmla="*/ 762000 w 2124075"/>
+            <a:gd name="connsiteY12" fmla="*/ 486122 h 809972"/>
+            <a:gd name="connsiteX13" fmla="*/ 714375 w 2124075"/>
+            <a:gd name="connsiteY13" fmla="*/ 428972 h 809972"/>
+            <a:gd name="connsiteX14" fmla="*/ 647700 w 2124075"/>
+            <a:gd name="connsiteY14" fmla="*/ 343247 h 809972"/>
+            <a:gd name="connsiteX15" fmla="*/ 600075 w 2124075"/>
+            <a:gd name="connsiteY15" fmla="*/ 276572 h 809972"/>
+            <a:gd name="connsiteX16" fmla="*/ 542925 w 2124075"/>
+            <a:gd name="connsiteY16" fmla="*/ 200372 h 809972"/>
+            <a:gd name="connsiteX17" fmla="*/ 514350 w 2124075"/>
+            <a:gd name="connsiteY17" fmla="*/ 171797 h 809972"/>
+            <a:gd name="connsiteX18" fmla="*/ 466725 w 2124075"/>
+            <a:gd name="connsiteY18" fmla="*/ 114647 h 809972"/>
+            <a:gd name="connsiteX19" fmla="*/ 409575 w 2124075"/>
+            <a:gd name="connsiteY19" fmla="*/ 76547 h 809972"/>
+            <a:gd name="connsiteX20" fmla="*/ 352425 w 2124075"/>
+            <a:gd name="connsiteY20" fmla="*/ 47972 h 809972"/>
+            <a:gd name="connsiteX21" fmla="*/ 209550 w 2124075"/>
+            <a:gd name="connsiteY21" fmla="*/ 28922 h 809972"/>
+            <a:gd name="connsiteX22" fmla="*/ 152400 w 2124075"/>
+            <a:gd name="connsiteY22" fmla="*/ 9872 h 809972"/>
+            <a:gd name="connsiteX23" fmla="*/ 0 w 2124075"/>
+            <a:gd name="connsiteY23" fmla="*/ 347 h 809972"/>
+          </a:gdLst>
+          <a:ahLst/>
+          <a:cxnLst>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX0" y="connsiteY0"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX1" y="connsiteY1"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX2" y="connsiteY2"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX3" y="connsiteY3"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX4" y="connsiteY4"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX5" y="connsiteY5"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX6" y="connsiteY6"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX7" y="connsiteY7"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX8" y="connsiteY8"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX9" y="connsiteY9"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX10" y="connsiteY10"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX11" y="connsiteY11"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX12" y="connsiteY12"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX13" y="connsiteY13"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX14" y="connsiteY14"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX15" y="connsiteY15"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX16" y="connsiteY16"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX17" y="connsiteY17"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX18" y="connsiteY18"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX19" y="connsiteY19"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX20" y="connsiteY20"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX21" y="connsiteY21"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX22" y="connsiteY22"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX23" y="connsiteY23"/>
+            </a:cxn>
+          </a:cxnLst>
+          <a:rect l="l" t="t" r="r" b="b"/>
+          <a:pathLst>
+            <a:path w="2124075" h="809972">
+              <a:moveTo>
+                <a:pt x="2124075" y="809972"/>
+              </a:moveTo>
+              <a:cubicBezTo>
+                <a:pt x="1997075" y="806797"/>
+                <a:pt x="1869977" y="806349"/>
+                <a:pt x="1743075" y="800447"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1733046" y="799981"/>
+                <a:pt x="1724240" y="793357"/>
+                <a:pt x="1714500" y="790922"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1635934" y="771280"/>
+                <a:pt x="1697221" y="791428"/>
+                <a:pt x="1628775" y="771872"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1577248" y="757150"/>
+                <a:pt x="1622290" y="764441"/>
+                <a:pt x="1552575" y="752822"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1423134" y="731249"/>
+                <a:pt x="1391638" y="740047"/>
+                <a:pt x="1209675" y="733772"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1196975" y="730597"/>
+                <a:pt x="1184488" y="726399"/>
+                <a:pt x="1171575" y="724247"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="1146326" y="720039"/>
+                <a:pt x="1120748" y="718105"/>
+                <a:pt x="1095375" y="714722"/>
+              </a:cubicBezTo>
+              <a:lnTo>
+                <a:pt x="1028700" y="705197"/>
+              </a:lnTo>
+              <a:cubicBezTo>
+                <a:pt x="1003300" y="692497"/>
+                <a:pt x="972580" y="687177"/>
+                <a:pt x="952500" y="667097"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="933450" y="648047"/>
+                <a:pt x="910294" y="632363"/>
+                <a:pt x="895350" y="609947"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="889000" y="600422"/>
+                <a:pt x="884915" y="588910"/>
+                <a:pt x="876300" y="581372"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="820073" y="532173"/>
+                <a:pt x="807876" y="554936"/>
+                <a:pt x="762000" y="486122"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="693927" y="384012"/>
+                <a:pt x="799938" y="538981"/>
+                <a:pt x="714375" y="428972"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="634624" y="326435"/>
+                <a:pt x="712574" y="408121"/>
+                <a:pt x="647700" y="343247"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="629688" y="289211"/>
+                <a:pt x="650297" y="336838"/>
+                <a:pt x="600075" y="276572"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="579749" y="252181"/>
+                <a:pt x="565376" y="222823"/>
+                <a:pt x="542925" y="200372"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="533400" y="190847"/>
+                <a:pt x="522974" y="182145"/>
+                <a:pt x="514350" y="171797"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="485385" y="137039"/>
+                <a:pt x="506269" y="145404"/>
+                <a:pt x="466725" y="114647"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="448653" y="100591"/>
+                <a:pt x="428625" y="89247"/>
+                <a:pt x="409575" y="76547"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="387634" y="61919"/>
+                <a:pt x="378715" y="52354"/>
+                <a:pt x="352425" y="47972"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="304857" y="40044"/>
+                <a:pt x="256535" y="40668"/>
+                <a:pt x="209550" y="28922"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="190069" y="24052"/>
+                <a:pt x="172325" y="12363"/>
+                <a:pt x="152400" y="9872"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="50996" y="-2803"/>
+                <a:pt x="101798" y="347"/>
+                <a:pt x="0" y="347"/>
+              </a:cubicBezTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:noFill/>
       </xdr:spPr>
       <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
         </a:lnRef>
-        <a:fillRef idx="0">
+        <a:fillRef idx="1">
           <a:schemeClr val="accent1"/>
         </a:fillRef>
         <a:effectRef idx="0">
           <a:schemeClr val="accent1"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
+          <a:schemeClr val="lt1"/>
         </a:fontRef>
       </xdr:style>
-    </xdr:cxnSp>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="tr-TR" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1533525</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>276208</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1790700</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="Serbest Form 11"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16411575" y="676258"/>
+          <a:ext cx="2057400" cy="2152667"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst>
+            <a:gd name="connsiteX0" fmla="*/ 0 w 2476500"/>
+            <a:gd name="connsiteY0" fmla="*/ 1866917 h 2152667"/>
+            <a:gd name="connsiteX1" fmla="*/ 95250 w 2476500"/>
+            <a:gd name="connsiteY1" fmla="*/ 1905017 h 2152667"/>
+            <a:gd name="connsiteX2" fmla="*/ 133350 w 2476500"/>
+            <a:gd name="connsiteY2" fmla="*/ 1924067 h 2152667"/>
+            <a:gd name="connsiteX3" fmla="*/ 1171575 w 2476500"/>
+            <a:gd name="connsiteY3" fmla="*/ 2152667 h 2152667"/>
+            <a:gd name="connsiteX4" fmla="*/ 1685925 w 2476500"/>
+            <a:gd name="connsiteY4" fmla="*/ 2076467 h 2152667"/>
+            <a:gd name="connsiteX5" fmla="*/ 1885950 w 2476500"/>
+            <a:gd name="connsiteY5" fmla="*/ 2019317 h 2152667"/>
+            <a:gd name="connsiteX6" fmla="*/ 1971675 w 2476500"/>
+            <a:gd name="connsiteY6" fmla="*/ 2000267 h 2152667"/>
+            <a:gd name="connsiteX7" fmla="*/ 2066925 w 2476500"/>
+            <a:gd name="connsiteY7" fmla="*/ 1943117 h 2152667"/>
+            <a:gd name="connsiteX8" fmla="*/ 2095500 w 2476500"/>
+            <a:gd name="connsiteY8" fmla="*/ 1914542 h 2152667"/>
+            <a:gd name="connsiteX9" fmla="*/ 2133600 w 2476500"/>
+            <a:gd name="connsiteY9" fmla="*/ 1885967 h 2152667"/>
+            <a:gd name="connsiteX10" fmla="*/ 2228850 w 2476500"/>
+            <a:gd name="connsiteY10" fmla="*/ 1743092 h 2152667"/>
+            <a:gd name="connsiteX11" fmla="*/ 2238375 w 2476500"/>
+            <a:gd name="connsiteY11" fmla="*/ 1714517 h 2152667"/>
+            <a:gd name="connsiteX12" fmla="*/ 2257425 w 2476500"/>
+            <a:gd name="connsiteY12" fmla="*/ 1676417 h 2152667"/>
+            <a:gd name="connsiteX13" fmla="*/ 2266950 w 2476500"/>
+            <a:gd name="connsiteY13" fmla="*/ 1638317 h 2152667"/>
+            <a:gd name="connsiteX14" fmla="*/ 2286000 w 2476500"/>
+            <a:gd name="connsiteY14" fmla="*/ 1600217 h 2152667"/>
+            <a:gd name="connsiteX15" fmla="*/ 2295525 w 2476500"/>
+            <a:gd name="connsiteY15" fmla="*/ 1571642 h 2152667"/>
+            <a:gd name="connsiteX16" fmla="*/ 2324100 w 2476500"/>
+            <a:gd name="connsiteY16" fmla="*/ 1514492 h 2152667"/>
+            <a:gd name="connsiteX17" fmla="*/ 2343150 w 2476500"/>
+            <a:gd name="connsiteY17" fmla="*/ 1447817 h 2152667"/>
+            <a:gd name="connsiteX18" fmla="*/ 2333625 w 2476500"/>
+            <a:gd name="connsiteY18" fmla="*/ 1038242 h 2152667"/>
+            <a:gd name="connsiteX19" fmla="*/ 2324100 w 2476500"/>
+            <a:gd name="connsiteY19" fmla="*/ 990617 h 2152667"/>
+            <a:gd name="connsiteX20" fmla="*/ 2314575 w 2476500"/>
+            <a:gd name="connsiteY20" fmla="*/ 933467 h 2152667"/>
+            <a:gd name="connsiteX21" fmla="*/ 2295525 w 2476500"/>
+            <a:gd name="connsiteY21" fmla="*/ 876317 h 2152667"/>
+            <a:gd name="connsiteX22" fmla="*/ 2276475 w 2476500"/>
+            <a:gd name="connsiteY22" fmla="*/ 800117 h 2152667"/>
+            <a:gd name="connsiteX23" fmla="*/ 2276475 w 2476500"/>
+            <a:gd name="connsiteY23" fmla="*/ 276242 h 2152667"/>
+            <a:gd name="connsiteX24" fmla="*/ 2314575 w 2476500"/>
+            <a:gd name="connsiteY24" fmla="*/ 209567 h 2152667"/>
+            <a:gd name="connsiteX25" fmla="*/ 2324100 w 2476500"/>
+            <a:gd name="connsiteY25" fmla="*/ 180992 h 2152667"/>
+            <a:gd name="connsiteX26" fmla="*/ 2352675 w 2476500"/>
+            <a:gd name="connsiteY26" fmla="*/ 142892 h 2152667"/>
+            <a:gd name="connsiteX27" fmla="*/ 2371725 w 2476500"/>
+            <a:gd name="connsiteY27" fmla="*/ 114317 h 2152667"/>
+            <a:gd name="connsiteX28" fmla="*/ 2428875 w 2476500"/>
+            <a:gd name="connsiteY28" fmla="*/ 57167 h 2152667"/>
+            <a:gd name="connsiteX29" fmla="*/ 2476500 w 2476500"/>
+            <a:gd name="connsiteY29" fmla="*/ 17 h 2152667"/>
+          </a:gdLst>
+          <a:ahLst/>
+          <a:cxnLst>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX0" y="connsiteY0"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX1" y="connsiteY1"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX2" y="connsiteY2"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX3" y="connsiteY3"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX4" y="connsiteY4"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX5" y="connsiteY5"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX6" y="connsiteY6"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX7" y="connsiteY7"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX8" y="connsiteY8"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX9" y="connsiteY9"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX10" y="connsiteY10"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX11" y="connsiteY11"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX12" y="connsiteY12"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX13" y="connsiteY13"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX14" y="connsiteY14"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX15" y="connsiteY15"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX16" y="connsiteY16"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX17" y="connsiteY17"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX18" y="connsiteY18"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX19" y="connsiteY19"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX20" y="connsiteY20"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX21" y="connsiteY21"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX22" y="connsiteY22"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX23" y="connsiteY23"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX24" y="connsiteY24"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX25" y="connsiteY25"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX26" y="connsiteY26"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX27" y="connsiteY27"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX28" y="connsiteY28"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX29" y="connsiteY29"/>
+            </a:cxn>
+          </a:cxnLst>
+          <a:rect l="l" t="t" r="r" b="b"/>
+          <a:pathLst>
+            <a:path w="2476500" h="2152667">
+              <a:moveTo>
+                <a:pt x="0" y="1866917"/>
+              </a:moveTo>
+              <a:cubicBezTo>
+                <a:pt x="31750" y="1879617"/>
+                <a:pt x="63819" y="1891547"/>
+                <a:pt x="95250" y="1905017"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="108301" y="1910610"/>
+                <a:pt x="119566" y="1920658"/>
+                <a:pt x="133350" y="1924067"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="937342" y="2122904"/>
+                <a:pt x="717446" y="2084548"/>
+                <a:pt x="1171575" y="2152667"/>
+              </a:cubicBezTo>
+              <a:lnTo>
+                <a:pt x="1685925" y="2076467"/>
+              </a:lnTo>
+              <a:cubicBezTo>
+                <a:pt x="1758673" y="2064733"/>
+                <a:pt x="1811898" y="2035773"/>
+                <a:pt x="1885950" y="2019317"/>
+              </a:cubicBezTo>
+              <a:lnTo>
+                <a:pt x="1971675" y="2000267"/>
+              </a:lnTo>
+              <a:cubicBezTo>
+                <a:pt x="2001740" y="1985235"/>
+                <a:pt x="2043937" y="1966105"/>
+                <a:pt x="2066925" y="1943117"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2076450" y="1933592"/>
+                <a:pt x="2085273" y="1923308"/>
+                <a:pt x="2095500" y="1914542"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2107553" y="1904211"/>
+                <a:pt x="2123346" y="1898086"/>
+                <a:pt x="2133600" y="1885967"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2146205" y="1871070"/>
+                <a:pt x="2211236" y="1778321"/>
+                <a:pt x="2228850" y="1743092"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2233340" y="1734112"/>
+                <a:pt x="2234420" y="1723745"/>
+                <a:pt x="2238375" y="1714517"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2243968" y="1701466"/>
+                <a:pt x="2252439" y="1689712"/>
+                <a:pt x="2257425" y="1676417"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2262022" y="1664160"/>
+                <a:pt x="2262353" y="1650574"/>
+                <a:pt x="2266950" y="1638317"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2271936" y="1625022"/>
+                <a:pt x="2280407" y="1613268"/>
+                <a:pt x="2286000" y="1600217"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2289955" y="1590989"/>
+                <a:pt x="2291447" y="1580817"/>
+                <a:pt x="2295525" y="1571642"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2304175" y="1552179"/>
+                <a:pt x="2315450" y="1533955"/>
+                <a:pt x="2324100" y="1514492"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2331908" y="1496923"/>
+                <a:pt x="2338826" y="1465115"/>
+                <a:pt x="2343150" y="1447817"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2339975" y="1311292"/>
+                <a:pt x="2339310" y="1174686"/>
+                <a:pt x="2333625" y="1038242"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2332951" y="1022067"/>
+                <a:pt x="2326996" y="1006545"/>
+                <a:pt x="2324100" y="990617"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2320645" y="971616"/>
+                <a:pt x="2319259" y="952203"/>
+                <a:pt x="2314575" y="933467"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2309705" y="913986"/>
+                <a:pt x="2299463" y="896008"/>
+                <a:pt x="2295525" y="876317"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2284031" y="818847"/>
+                <a:pt x="2291120" y="844051"/>
+                <a:pt x="2276475" y="800117"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2255217" y="587540"/>
+                <a:pt x="2255100" y="625360"/>
+                <a:pt x="2276475" y="276242"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2277640" y="257213"/>
+                <a:pt x="2306196" y="226326"/>
+                <a:pt x="2314575" y="209567"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2319065" y="200587"/>
+                <a:pt x="2319119" y="189709"/>
+                <a:pt x="2324100" y="180992"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2331976" y="167209"/>
+                <a:pt x="2343448" y="155810"/>
+                <a:pt x="2352675" y="142892"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2359329" y="133577"/>
+                <a:pt x="2364120" y="122873"/>
+                <a:pt x="2371725" y="114317"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2389623" y="94181"/>
+                <a:pt x="2413931" y="79583"/>
+                <a:pt x="2428875" y="57167"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="2468736" y="-2625"/>
+                <a:pt x="2444080" y="17"/>
+                <a:pt x="2476500" y="17"/>
+              </a:cubicBezTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="tr-TR" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -687,8 +1909,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr defaultColWidth="27" defaultRowHeight="31.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="34.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
@@ -715,15 +1940,15 @@
     </row>
     <row r="2" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="3" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
@@ -731,7 +1956,7 @@
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>13</v>
@@ -743,7 +1968,7 @@
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="3" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
@@ -771,7 +1996,7 @@
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
@@ -786,30 +2011,122 @@
       <c r="C5" s="9" t="s">
         <v>17</v>
       </c>
+      <c r="E5" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="G5" s="1" t="s">
         <v>12</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I6" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I7" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I8" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I9" s="1"/>
+      <c r="A9" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="3:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>